<commit_message>
feat: split belastingen into R&O, add opmerking fields and CMMI-aligned schaal
- Split "Belastingen" platform into "belastingen" and "ro" (R&O)
- Add per-question opmerking (toelichting) textarea and a general
  toelichting field per platform-meting, wired into the invulformulier
- Align 1-5 schaal labels/descriptions with CMMI (Initial to Optimizing)
  and show a visible legend on the invulformulier
- Add two proces-vragen on being a "partner van betekenis" for
  productontwikkeling and dienstverlening
- Escape user-controlled text in renderInvullen to prevent stored XSS
  via imported data
- Deduplicate CONFIG: generate-xlsx.cjs -> generate-xlsx.mjs importing
  from js/config.js instead of a hand-copied duplicate
- Update Playwright suite for the new platform/question counts and add
  coverage for the schaal legend and opmerking persistence
</commit_message>
<xml_diff>
--- a/GVPRLG-Volwassenheidsmeting-v2.xlsx
+++ b/GVPRLG-Volwassenheidsmeting-v2.xlsx
@@ -400,7 +400,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G61"/>
+  <dimension ref="A1:G86"/>
   <cols>
     <col min="1" max="1" width="22.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -781,16 +781,16 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>Burgerzaken</v>
+        <v>Belastingen</v>
       </c>
       <c r="B17" t="str">
-        <v/>
+        <v>Proces</v>
       </c>
       <c r="C17" t="str">
-        <v/>
+        <v>partner-productontwikkeling</v>
       </c>
       <c r="D17" t="str">
-        <v/>
+        <v>PinkRoccade is een partner van betekenis: de productontwikkeling sluit voldoende aan bij de wensen en eisen die vanuit de markt (gemeenten) worden gesteld</v>
       </c>
       <c r="E17" t="str">
         <v/>
@@ -804,19 +804,19 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>Burgerzaken</v>
+        <v>Belastingen</v>
       </c>
       <c r="B18" t="str">
-        <v>Techniek</v>
+        <v>Proces</v>
       </c>
       <c r="C18" t="str">
-        <v>common-ground-standaarden</v>
+        <v>partner-dienstverlening</v>
       </c>
       <c r="D18" t="str">
-        <v>De producten voldoen aan Common Ground-principes en open standaarden (API-first, ZGW-API's, iConnect, scheiding data/logica)</v>
+        <v>PinkRoccade is een partner van betekenis: de dienstverlening sluit voldoende aan bij de wensen en eisen die vanuit de markt (gemeenten) worden gesteld</v>
       </c>
       <c r="E18" t="str">
-        <v>Open</v>
+        <v/>
       </c>
       <c r="F18" t="str">
         <v/>
@@ -827,19 +827,19 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>Burgerzaken</v>
+        <v>R&amp;O</v>
       </c>
       <c r="B19" t="str">
-        <v>Techniek</v>
+        <v/>
       </c>
       <c r="C19" t="str">
-        <v>cloud-data</v>
+        <v/>
       </c>
       <c r="D19" t="str">
-        <v>De producten zijn volwaardige SaaS-oplossingen met datagedreven werken: data via API's beschikbaar voor analyse en veilig deelbaar over overheidslagen</v>
+        <v/>
       </c>
       <c r="E19" t="str">
-        <v>Cloud</v>
+        <v/>
       </c>
       <c r="F19" t="str">
         <v/>
@@ -850,19 +850,19 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>Burgerzaken</v>
+        <v>R&amp;O</v>
       </c>
       <c r="B20" t="str">
         <v>Techniek</v>
       </c>
       <c r="C20" t="str">
-        <v>ai-integratie</v>
+        <v>common-ground-standaarden</v>
       </c>
       <c r="D20" t="str">
-        <v>AI is concreet en bruikbaar onderdeel van de productportfolio (werkende functionaliteit, niet alleen visie) en hierover zijn risicoanalyses uitgevoerd en een AI-act assessment van beschikbaar</v>
+        <v>De producten voldoen aan Common Ground-principes en open standaarden (API-first, ZGW-API's, iConnect, scheiding data/logica)</v>
       </c>
       <c r="E20" t="str">
-        <v>AI</v>
+        <v>Open</v>
       </c>
       <c r="F20" t="str">
         <v/>
@@ -873,19 +873,19 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>Burgerzaken</v>
+        <v>R&amp;O</v>
       </c>
       <c r="B21" t="str">
         <v>Techniek</v>
       </c>
       <c r="C21" t="str">
-        <v>digitale-weerbaarheid</v>
+        <v>cloud-data</v>
       </c>
       <c r="D21" t="str">
-        <v>De producten voldoen aan actuele security-eisen (BIO, NIS2, pentesting) en verminderen leveranciersafhankelijkheid</v>
+        <v>De producten zijn volwaardige SaaS-oplossingen met datagedreven werken: data via API's beschikbaar voor analyse en veilig deelbaar over overheidslagen</v>
       </c>
       <c r="E21" t="str">
-        <v>Digitale weerbaarheid en autonomie</v>
+        <v>Cloud</v>
       </c>
       <c r="F21" t="str">
         <v/>
@@ -896,19 +896,19 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>Burgerzaken</v>
+        <v>R&amp;O</v>
       </c>
       <c r="B22" t="str">
-        <v>Mens</v>
+        <v>Techniek</v>
       </c>
       <c r="C22" t="str">
-        <v>capaciteit-kennis</v>
+        <v>ai-integratie</v>
       </c>
       <c r="D22" t="str">
-        <v>De personele capaciteit (aantal en kennisniveau) is op orde om producten te ondersteunen en door te ontwikkelen en heeft een meerjaars forecast</v>
+        <v>AI is concreet en bruikbaar onderdeel van de productportfolio (werkende functionaliteit, niet alleen visie) en hierover zijn risicoanalyses uitgevoerd en een AI-act assessment van beschikbaar</v>
       </c>
       <c r="E22" t="str">
-        <v/>
+        <v>AI</v>
       </c>
       <c r="F22" t="str">
         <v/>
@@ -919,19 +919,19 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>Burgerzaken</v>
+        <v>R&amp;O</v>
       </c>
       <c r="B23" t="str">
-        <v>Mens</v>
+        <v>Techniek</v>
       </c>
       <c r="C23" t="str">
-        <v>digitaal-vakmanschap</v>
+        <v>digitale-weerbaarheid</v>
       </c>
       <c r="D23" t="str">
-        <v>PinkRoccade investeert aantoonbaar in kennisontwikkeling (nieuwe technologieën, AI, Common Ground) en ondersteunt gemeenten hierbij</v>
+        <v>De producten voldoen aan actuele security-eisen (BIO, NIS2, pentesting) en verminderen leveranciersafhankelijkheid</v>
       </c>
       <c r="E23" t="str">
-        <v>Digitaal vakmanschap</v>
+        <v>Digitale weerbaarheid en autonomie</v>
       </c>
       <c r="F23" t="str">
         <v/>
@@ -942,16 +942,16 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>Burgerzaken</v>
+        <v>R&amp;O</v>
       </c>
       <c r="B24" t="str">
         <v>Mens</v>
       </c>
       <c r="C24" t="str">
-        <v>klantbetrokkenheid</v>
+        <v>capaciteit-kennis</v>
       </c>
       <c r="D24" t="str">
-        <v>Gebruikers worden structureel betrokken bij doorontwikkeling (co-creatie, klankbordgroepen, roadmap-invloed) en de betrokkenheid wordt op kwaliteit en kwantiteit periodiek geëvalueerd</v>
+        <v>De personele capaciteit (aantal en kennisniveau) is op orde om producten te ondersteunen en door te ontwikkelen en heeft een meerjaars forecast</v>
       </c>
       <c r="E24" t="str">
         <v/>
@@ -965,19 +965,19 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>Burgerzaken</v>
+        <v>R&amp;O</v>
       </c>
       <c r="B25" t="str">
         <v>Mens</v>
       </c>
       <c r="C25" t="str">
-        <v>opleiding-continuiteit</v>
+        <v>digitaal-vakmanschap</v>
       </c>
       <c r="D25" t="str">
-        <v>Training, documentatie en support zijn op orde; kennisborging is geborgd en niet afhankelijk van individuen</v>
+        <v>PinkRoccade investeert aantoonbaar in kennisontwikkeling (nieuwe technologieën, AI, Common Ground) en ondersteunt gemeenten hierbij</v>
       </c>
       <c r="E25" t="str">
-        <v/>
+        <v>Digitaal vakmanschap</v>
       </c>
       <c r="F25" t="str">
         <v/>
@@ -988,16 +988,16 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>Burgerzaken</v>
+        <v>R&amp;O</v>
       </c>
       <c r="B26" t="str">
-        <v>Proces</v>
+        <v>Mens</v>
       </c>
       <c r="C26" t="str">
-        <v>dienstverlening-nps</v>
+        <v>klantbetrokkenheid</v>
       </c>
       <c r="D26" t="str">
-        <v>De dienstverlening is uniform tussen businessunits; NPS en klanttevredenheid worden structureel gemeten en vertaald naar verbeteracties en gepubliceerd</v>
+        <v>Gebruikers worden structureel betrokken bij doorontwikkeling (co-creatie, klankbordgroepen, roadmap-invloed) en de betrokkenheid wordt op kwaliteit en kwantiteit periodiek geëvalueerd</v>
       </c>
       <c r="E26" t="str">
         <v/>
@@ -1011,16 +1011,16 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>Burgerzaken</v>
+        <v>R&amp;O</v>
       </c>
       <c r="B27" t="str">
-        <v>Proces</v>
+        <v>Mens</v>
       </c>
       <c r="C27" t="str">
-        <v>release-incident</v>
+        <v>opleiding-continuiteit</v>
       </c>
       <c r="D27" t="str">
-        <v>Releases zijn voorspelbaar en goed gecommuniceerd; incidenten worden snel en transparant conform SLA afgehandeld</v>
+        <v>Training, documentatie en support zijn op orde; kennisborging is geborgd en niet afhankelijk van individuen</v>
       </c>
       <c r="E27" t="str">
         <v/>
@@ -1034,16 +1034,16 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>Burgerzaken</v>
+        <v>R&amp;O</v>
       </c>
       <c r="B28" t="str">
         <v>Proces</v>
       </c>
       <c r="C28" t="str">
-        <v>roadmap-transparantie</v>
+        <v>dienstverlening-nps</v>
       </c>
       <c r="D28" t="str">
-        <v>De productroadmap is transparant, realistisch en sluit aan bij NDS-prioriteiten en gemeentelijke behoeften</v>
+        <v>De dienstverlening is uniform tussen businessunits; NPS en klanttevredenheid worden structureel gemeten en vertaald naar verbeteracties en gepubliceerd</v>
       </c>
       <c r="E28" t="str">
         <v/>
@@ -1057,19 +1057,19 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>Burgerzaken</v>
+        <v>R&amp;O</v>
       </c>
       <c r="B29" t="str">
         <v>Proces</v>
       </c>
       <c r="C29" t="str">
-        <v>burgers-ondernemers-centraal</v>
+        <v>release-incident</v>
       </c>
       <c r="D29" t="str">
-        <v>De producten stellen gemeenten in staat burgers en ondernemers als één overheid te bedienen met geïntegreerde digitale dienstverlening</v>
+        <v>Releases zijn voorspelbaar en goed gecommuniceerd; incidenten worden snel en transparant conform SLA afgehandeld</v>
       </c>
       <c r="E29" t="str">
-        <v>Burgers en ondernemers centraal</v>
+        <v/>
       </c>
       <c r="F29" t="str">
         <v/>
@@ -1080,16 +1080,16 @@
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>Burgerzaken</v>
+        <v>R&amp;O</v>
       </c>
       <c r="B30" t="str">
         <v>Proces</v>
       </c>
       <c r="C30" t="str">
-        <v>prijsbeleid</v>
+        <v>roadmap-transparantie</v>
       </c>
       <c r="D30" t="str">
-        <v>Prijsbeleid (inclusief offertes) is uitlegbaar en marktconform en hanteert een voorspelbaar proces</v>
+        <v>De productroadmap is transparant, realistisch en sluit aan bij NDS-prioriteiten en gemeentelijke behoeften</v>
       </c>
       <c r="E30" t="str">
         <v/>
@@ -1103,19 +1103,19 @@
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>Burgerzaken</v>
+        <v>R&amp;O</v>
       </c>
       <c r="B31" t="str">
         <v>Proces</v>
       </c>
       <c r="C31" t="str">
-        <v>lifecyclemanagement</v>
+        <v>burgers-ondernemers-centraal</v>
       </c>
       <c r="D31" t="str">
-        <v>Lifecyclemanagement volgt de afspraken van de uitvloeiingsregeling</v>
+        <v>De producten stellen gemeenten in staat burgers en ondernemers als één overheid te bedienen met geïntegreerde digitale dienstverlening</v>
       </c>
       <c r="E31" t="str">
-        <v/>
+        <v>Burgers en ondernemers centraal</v>
       </c>
       <c r="F31" t="str">
         <v/>
@@ -1126,16 +1126,16 @@
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>Sociaal Domein</v>
+        <v>R&amp;O</v>
       </c>
       <c r="B32" t="str">
-        <v/>
+        <v>Proces</v>
       </c>
       <c r="C32" t="str">
-        <v/>
+        <v>prijsbeleid</v>
       </c>
       <c r="D32" t="str">
-        <v/>
+        <v>Prijsbeleid (inclusief offertes) is uitlegbaar en marktconform en hanteert een voorspelbaar proces</v>
       </c>
       <c r="E32" t="str">
         <v/>
@@ -1149,19 +1149,19 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>Sociaal Domein</v>
+        <v>R&amp;O</v>
       </c>
       <c r="B33" t="str">
-        <v>Techniek</v>
+        <v>Proces</v>
       </c>
       <c r="C33" t="str">
-        <v>common-ground-standaarden</v>
+        <v>lifecyclemanagement</v>
       </c>
       <c r="D33" t="str">
-        <v>De producten voldoen aan Common Ground-principes en open standaarden (API-first, ZGW-API's, iConnect, scheiding data/logica)</v>
+        <v>Lifecyclemanagement volgt de afspraken van de uitvloeiingsregeling</v>
       </c>
       <c r="E33" t="str">
-        <v>Open</v>
+        <v/>
       </c>
       <c r="F33" t="str">
         <v/>
@@ -1172,19 +1172,19 @@
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>Sociaal Domein</v>
+        <v>R&amp;O</v>
       </c>
       <c r="B34" t="str">
-        <v>Techniek</v>
+        <v>Proces</v>
       </c>
       <c r="C34" t="str">
-        <v>cloud-data</v>
+        <v>partner-productontwikkeling</v>
       </c>
       <c r="D34" t="str">
-        <v>De producten zijn volwaardige SaaS-oplossingen met datagedreven werken: data via API's beschikbaar voor analyse en veilig deelbaar over overheidslagen</v>
+        <v>PinkRoccade is een partner van betekenis: de productontwikkeling sluit voldoende aan bij de wensen en eisen die vanuit de markt (gemeenten) worden gesteld</v>
       </c>
       <c r="E34" t="str">
-        <v>Cloud</v>
+        <v/>
       </c>
       <c r="F34" t="str">
         <v/>
@@ -1195,19 +1195,19 @@
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>Sociaal Domein</v>
+        <v>R&amp;O</v>
       </c>
       <c r="B35" t="str">
-        <v>Techniek</v>
+        <v>Proces</v>
       </c>
       <c r="C35" t="str">
-        <v>ai-integratie</v>
+        <v>partner-dienstverlening</v>
       </c>
       <c r="D35" t="str">
-        <v>AI is concreet en bruikbaar onderdeel van de productportfolio (werkende functionaliteit, niet alleen visie) en hierover zijn risicoanalyses uitgevoerd en een AI-act assessment van beschikbaar</v>
+        <v>PinkRoccade is een partner van betekenis: de dienstverlening sluit voldoende aan bij de wensen en eisen die vanuit de markt (gemeenten) worden gesteld</v>
       </c>
       <c r="E35" t="str">
-        <v>AI</v>
+        <v/>
       </c>
       <c r="F35" t="str">
         <v/>
@@ -1218,19 +1218,19 @@
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>Sociaal Domein</v>
+        <v>Burgerzaken</v>
       </c>
       <c r="B36" t="str">
-        <v>Techniek</v>
+        <v/>
       </c>
       <c r="C36" t="str">
-        <v>digitale-weerbaarheid</v>
+        <v/>
       </c>
       <c r="D36" t="str">
-        <v>De producten voldoen aan actuele security-eisen (BIO, NIS2, pentesting) en verminderen leveranciersafhankelijkheid</v>
+        <v/>
       </c>
       <c r="E36" t="str">
-        <v>Digitale weerbaarheid en autonomie</v>
+        <v/>
       </c>
       <c r="F36" t="str">
         <v/>
@@ -1241,19 +1241,19 @@
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>Sociaal Domein</v>
+        <v>Burgerzaken</v>
       </c>
       <c r="B37" t="str">
-        <v>Mens</v>
+        <v>Techniek</v>
       </c>
       <c r="C37" t="str">
-        <v>capaciteit-kennis</v>
+        <v>common-ground-standaarden</v>
       </c>
       <c r="D37" t="str">
-        <v>De personele capaciteit (aantal en kennisniveau) is op orde om producten te ondersteunen en door te ontwikkelen en heeft een meerjaars forecast</v>
+        <v>De producten voldoen aan Common Ground-principes en open standaarden (API-first, ZGW-API's, iConnect, scheiding data/logica)</v>
       </c>
       <c r="E37" t="str">
-        <v/>
+        <v>Open</v>
       </c>
       <c r="F37" t="str">
         <v/>
@@ -1264,19 +1264,19 @@
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>Sociaal Domein</v>
+        <v>Burgerzaken</v>
       </c>
       <c r="B38" t="str">
-        <v>Mens</v>
+        <v>Techniek</v>
       </c>
       <c r="C38" t="str">
-        <v>digitaal-vakmanschap</v>
+        <v>cloud-data</v>
       </c>
       <c r="D38" t="str">
-        <v>PinkRoccade investeert aantoonbaar in kennisontwikkeling (nieuwe technologieën, AI, Common Ground) en ondersteunt gemeenten hierbij</v>
+        <v>De producten zijn volwaardige SaaS-oplossingen met datagedreven werken: data via API's beschikbaar voor analyse en veilig deelbaar over overheidslagen</v>
       </c>
       <c r="E38" t="str">
-        <v>Digitaal vakmanschap</v>
+        <v>Cloud</v>
       </c>
       <c r="F38" t="str">
         <v/>
@@ -1287,19 +1287,19 @@
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>Sociaal Domein</v>
+        <v>Burgerzaken</v>
       </c>
       <c r="B39" t="str">
-        <v>Mens</v>
+        <v>Techniek</v>
       </c>
       <c r="C39" t="str">
-        <v>klantbetrokkenheid</v>
+        <v>ai-integratie</v>
       </c>
       <c r="D39" t="str">
-        <v>Gebruikers worden structureel betrokken bij doorontwikkeling (co-creatie, klankbordgroepen, roadmap-invloed) en de betrokkenheid wordt op kwaliteit en kwantiteit periodiek geëvalueerd</v>
+        <v>AI is concreet en bruikbaar onderdeel van de productportfolio (werkende functionaliteit, niet alleen visie) en hierover zijn risicoanalyses uitgevoerd en een AI-act assessment van beschikbaar</v>
       </c>
       <c r="E39" t="str">
-        <v/>
+        <v>AI</v>
       </c>
       <c r="F39" t="str">
         <v/>
@@ -1310,19 +1310,19 @@
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>Sociaal Domein</v>
+        <v>Burgerzaken</v>
       </c>
       <c r="B40" t="str">
-        <v>Mens</v>
+        <v>Techniek</v>
       </c>
       <c r="C40" t="str">
-        <v>opleiding-continuiteit</v>
+        <v>digitale-weerbaarheid</v>
       </c>
       <c r="D40" t="str">
-        <v>Training, documentatie en support zijn op orde; kennisborging is geborgd en niet afhankelijk van individuen</v>
+        <v>De producten voldoen aan actuele security-eisen (BIO, NIS2, pentesting) en verminderen leveranciersafhankelijkheid</v>
       </c>
       <c r="E40" t="str">
-        <v/>
+        <v>Digitale weerbaarheid en autonomie</v>
       </c>
       <c r="F40" t="str">
         <v/>
@@ -1333,16 +1333,16 @@
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>Sociaal Domein</v>
+        <v>Burgerzaken</v>
       </c>
       <c r="B41" t="str">
-        <v>Proces</v>
+        <v>Mens</v>
       </c>
       <c r="C41" t="str">
-        <v>dienstverlening-nps</v>
+        <v>capaciteit-kennis</v>
       </c>
       <c r="D41" t="str">
-        <v>De dienstverlening is uniform tussen businessunits; NPS en klanttevredenheid worden structureel gemeten en vertaald naar verbeteracties en gepubliceerd</v>
+        <v>De personele capaciteit (aantal en kennisniveau) is op orde om producten te ondersteunen en door te ontwikkelen en heeft een meerjaars forecast</v>
       </c>
       <c r="E41" t="str">
         <v/>
@@ -1356,19 +1356,19 @@
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>Sociaal Domein</v>
+        <v>Burgerzaken</v>
       </c>
       <c r="B42" t="str">
-        <v>Proces</v>
+        <v>Mens</v>
       </c>
       <c r="C42" t="str">
-        <v>release-incident</v>
+        <v>digitaal-vakmanschap</v>
       </c>
       <c r="D42" t="str">
-        <v>Releases zijn voorspelbaar en goed gecommuniceerd; incidenten worden snel en transparant conform SLA afgehandeld</v>
+        <v>PinkRoccade investeert aantoonbaar in kennisontwikkeling (nieuwe technologieën, AI, Common Ground) en ondersteunt gemeenten hierbij</v>
       </c>
       <c r="E42" t="str">
-        <v/>
+        <v>Digitaal vakmanschap</v>
       </c>
       <c r="F42" t="str">
         <v/>
@@ -1379,16 +1379,16 @@
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>Sociaal Domein</v>
+        <v>Burgerzaken</v>
       </c>
       <c r="B43" t="str">
-        <v>Proces</v>
+        <v>Mens</v>
       </c>
       <c r="C43" t="str">
-        <v>roadmap-transparantie</v>
+        <v>klantbetrokkenheid</v>
       </c>
       <c r="D43" t="str">
-        <v>De productroadmap is transparant, realistisch en sluit aan bij NDS-prioriteiten en gemeentelijke behoeften</v>
+        <v>Gebruikers worden structureel betrokken bij doorontwikkeling (co-creatie, klankbordgroepen, roadmap-invloed) en de betrokkenheid wordt op kwaliteit en kwantiteit periodiek geëvalueerd</v>
       </c>
       <c r="E43" t="str">
         <v/>
@@ -1402,19 +1402,19 @@
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>Sociaal Domein</v>
+        <v>Burgerzaken</v>
       </c>
       <c r="B44" t="str">
-        <v>Proces</v>
+        <v>Mens</v>
       </c>
       <c r="C44" t="str">
-        <v>burgers-ondernemers-centraal</v>
+        <v>opleiding-continuiteit</v>
       </c>
       <c r="D44" t="str">
-        <v>De producten stellen gemeenten in staat burgers en ondernemers als één overheid te bedienen met geïntegreerde digitale dienstverlening</v>
+        <v>Training, documentatie en support zijn op orde; kennisborging is geborgd en niet afhankelijk van individuen</v>
       </c>
       <c r="E44" t="str">
-        <v>Burgers en ondernemers centraal</v>
+        <v/>
       </c>
       <c r="F44" t="str">
         <v/>
@@ -1425,16 +1425,16 @@
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>Sociaal Domein</v>
+        <v>Burgerzaken</v>
       </c>
       <c r="B45" t="str">
         <v>Proces</v>
       </c>
       <c r="C45" t="str">
-        <v>prijsbeleid</v>
+        <v>dienstverlening-nps</v>
       </c>
       <c r="D45" t="str">
-        <v>Prijsbeleid (inclusief offertes) is uitlegbaar en marktconform en hanteert een voorspelbaar proces</v>
+        <v>De dienstverlening is uniform tussen businessunits; NPS en klanttevredenheid worden structureel gemeten en vertaald naar verbeteracties en gepubliceerd</v>
       </c>
       <c r="E45" t="str">
         <v/>
@@ -1448,16 +1448,16 @@
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>Sociaal Domein</v>
+        <v>Burgerzaken</v>
       </c>
       <c r="B46" t="str">
         <v>Proces</v>
       </c>
       <c r="C46" t="str">
-        <v>lifecyclemanagement</v>
+        <v>release-incident</v>
       </c>
       <c r="D46" t="str">
-        <v>Lifecyclemanagement volgt de afspraken van de uitvloeiingsregeling</v>
+        <v>Releases zijn voorspelbaar en goed gecommuniceerd; incidenten worden snel en transparant conform SLA afgehandeld</v>
       </c>
       <c r="E46" t="str">
         <v/>
@@ -1471,16 +1471,16 @@
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>Informatievoorziening</v>
+        <v>Burgerzaken</v>
       </c>
       <c r="B47" t="str">
-        <v/>
+        <v>Proces</v>
       </c>
       <c r="C47" t="str">
-        <v/>
+        <v>roadmap-transparantie</v>
       </c>
       <c r="D47" t="str">
-        <v/>
+        <v>De productroadmap is transparant, realistisch en sluit aan bij NDS-prioriteiten en gemeentelijke behoeften</v>
       </c>
       <c r="E47" t="str">
         <v/>
@@ -1494,19 +1494,19 @@
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>Informatievoorziening</v>
+        <v>Burgerzaken</v>
       </c>
       <c r="B48" t="str">
-        <v>Techniek</v>
+        <v>Proces</v>
       </c>
       <c r="C48" t="str">
-        <v>common-ground-standaarden</v>
+        <v>burgers-ondernemers-centraal</v>
       </c>
       <c r="D48" t="str">
-        <v>De producten voldoen aan Common Ground-principes en open standaarden (API-first, ZGW-API's, iConnect, scheiding data/logica)</v>
+        <v>De producten stellen gemeenten in staat burgers en ondernemers als één overheid te bedienen met geïntegreerde digitale dienstverlening</v>
       </c>
       <c r="E48" t="str">
-        <v>Open</v>
+        <v>Burgers en ondernemers centraal</v>
       </c>
       <c r="F48" t="str">
         <v/>
@@ -1517,19 +1517,19 @@
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>Informatievoorziening</v>
+        <v>Burgerzaken</v>
       </c>
       <c r="B49" t="str">
-        <v>Techniek</v>
+        <v>Proces</v>
       </c>
       <c r="C49" t="str">
-        <v>cloud-data</v>
+        <v>prijsbeleid</v>
       </c>
       <c r="D49" t="str">
-        <v>De producten zijn volwaardige SaaS-oplossingen met datagedreven werken: data via API's beschikbaar voor analyse en veilig deelbaar over overheidslagen</v>
+        <v>Prijsbeleid (inclusief offertes) is uitlegbaar en marktconform en hanteert een voorspelbaar proces</v>
       </c>
       <c r="E49" t="str">
-        <v>Cloud</v>
+        <v/>
       </c>
       <c r="F49" t="str">
         <v/>
@@ -1540,19 +1540,19 @@
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>Informatievoorziening</v>
+        <v>Burgerzaken</v>
       </c>
       <c r="B50" t="str">
-        <v>Techniek</v>
+        <v>Proces</v>
       </c>
       <c r="C50" t="str">
-        <v>ai-integratie</v>
+        <v>lifecyclemanagement</v>
       </c>
       <c r="D50" t="str">
-        <v>AI is concreet en bruikbaar onderdeel van de productportfolio (werkende functionaliteit, niet alleen visie) en hierover zijn risicoanalyses uitgevoerd en een AI-act assessment van beschikbaar</v>
+        <v>Lifecyclemanagement volgt de afspraken van de uitvloeiingsregeling</v>
       </c>
       <c r="E50" t="str">
-        <v>AI</v>
+        <v/>
       </c>
       <c r="F50" t="str">
         <v/>
@@ -1563,19 +1563,19 @@
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>Informatievoorziening</v>
+        <v>Burgerzaken</v>
       </c>
       <c r="B51" t="str">
-        <v>Techniek</v>
+        <v>Proces</v>
       </c>
       <c r="C51" t="str">
-        <v>digitale-weerbaarheid</v>
+        <v>partner-productontwikkeling</v>
       </c>
       <c r="D51" t="str">
-        <v>De producten voldoen aan actuele security-eisen (BIO, NIS2, pentesting) en verminderen leveranciersafhankelijkheid</v>
+        <v>PinkRoccade is een partner van betekenis: de productontwikkeling sluit voldoende aan bij de wensen en eisen die vanuit de markt (gemeenten) worden gesteld</v>
       </c>
       <c r="E51" t="str">
-        <v>Digitale weerbaarheid en autonomie</v>
+        <v/>
       </c>
       <c r="F51" t="str">
         <v/>
@@ -1586,16 +1586,16 @@
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>Informatievoorziening</v>
+        <v>Burgerzaken</v>
       </c>
       <c r="B52" t="str">
-        <v>Mens</v>
+        <v>Proces</v>
       </c>
       <c r="C52" t="str">
-        <v>capaciteit-kennis</v>
+        <v>partner-dienstverlening</v>
       </c>
       <c r="D52" t="str">
-        <v>De personele capaciteit (aantal en kennisniveau) is op orde om producten te ondersteunen en door te ontwikkelen en heeft een meerjaars forecast</v>
+        <v>PinkRoccade is een partner van betekenis: de dienstverlening sluit voldoende aan bij de wensen en eisen die vanuit de markt (gemeenten) worden gesteld</v>
       </c>
       <c r="E52" t="str">
         <v/>
@@ -1609,19 +1609,19 @@
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>Informatievoorziening</v>
+        <v>Sociaal Domein</v>
       </c>
       <c r="B53" t="str">
-        <v>Mens</v>
+        <v/>
       </c>
       <c r="C53" t="str">
-        <v>digitaal-vakmanschap</v>
+        <v/>
       </c>
       <c r="D53" t="str">
-        <v>PinkRoccade investeert aantoonbaar in kennisontwikkeling (nieuwe technologieën, AI, Common Ground) en ondersteunt gemeenten hierbij</v>
+        <v/>
       </c>
       <c r="E53" t="str">
-        <v>Digitaal vakmanschap</v>
+        <v/>
       </c>
       <c r="F53" t="str">
         <v/>
@@ -1632,19 +1632,19 @@
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>Informatievoorziening</v>
+        <v>Sociaal Domein</v>
       </c>
       <c r="B54" t="str">
-        <v>Mens</v>
+        <v>Techniek</v>
       </c>
       <c r="C54" t="str">
-        <v>klantbetrokkenheid</v>
+        <v>common-ground-standaarden</v>
       </c>
       <c r="D54" t="str">
-        <v>Gebruikers worden structureel betrokken bij doorontwikkeling (co-creatie, klankbordgroepen, roadmap-invloed) en de betrokkenheid wordt op kwaliteit en kwantiteit periodiek geëvalueerd</v>
+        <v>De producten voldoen aan Common Ground-principes en open standaarden (API-first, ZGW-API's, iConnect, scheiding data/logica)</v>
       </c>
       <c r="E54" t="str">
-        <v/>
+        <v>Open</v>
       </c>
       <c r="F54" t="str">
         <v/>
@@ -1655,19 +1655,19 @@
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>Informatievoorziening</v>
+        <v>Sociaal Domein</v>
       </c>
       <c r="B55" t="str">
-        <v>Mens</v>
+        <v>Techniek</v>
       </c>
       <c r="C55" t="str">
-        <v>opleiding-continuiteit</v>
+        <v>cloud-data</v>
       </c>
       <c r="D55" t="str">
-        <v>Training, documentatie en support zijn op orde; kennisborging is geborgd en niet afhankelijk van individuen</v>
+        <v>De producten zijn volwaardige SaaS-oplossingen met datagedreven werken: data via API's beschikbaar voor analyse en veilig deelbaar over overheidslagen</v>
       </c>
       <c r="E55" t="str">
-        <v/>
+        <v>Cloud</v>
       </c>
       <c r="F55" t="str">
         <v/>
@@ -1678,19 +1678,19 @@
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>Informatievoorziening</v>
+        <v>Sociaal Domein</v>
       </c>
       <c r="B56" t="str">
-        <v>Proces</v>
+        <v>Techniek</v>
       </c>
       <c r="C56" t="str">
-        <v>dienstverlening-nps</v>
+        <v>ai-integratie</v>
       </c>
       <c r="D56" t="str">
-        <v>De dienstverlening is uniform tussen businessunits; NPS en klanttevredenheid worden structureel gemeten en vertaald naar verbeteracties en gepubliceerd</v>
+        <v>AI is concreet en bruikbaar onderdeel van de productportfolio (werkende functionaliteit, niet alleen visie) en hierover zijn risicoanalyses uitgevoerd en een AI-act assessment van beschikbaar</v>
       </c>
       <c r="E56" t="str">
-        <v/>
+        <v>AI</v>
       </c>
       <c r="F56" t="str">
         <v/>
@@ -1701,19 +1701,19 @@
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>Informatievoorziening</v>
+        <v>Sociaal Domein</v>
       </c>
       <c r="B57" t="str">
-        <v>Proces</v>
+        <v>Techniek</v>
       </c>
       <c r="C57" t="str">
-        <v>release-incident</v>
+        <v>digitale-weerbaarheid</v>
       </c>
       <c r="D57" t="str">
-        <v>Releases zijn voorspelbaar en goed gecommuniceerd; incidenten worden snel en transparant conform SLA afgehandeld</v>
+        <v>De producten voldoen aan actuele security-eisen (BIO, NIS2, pentesting) en verminderen leveranciersafhankelijkheid</v>
       </c>
       <c r="E57" t="str">
-        <v/>
+        <v>Digitale weerbaarheid en autonomie</v>
       </c>
       <c r="F57" t="str">
         <v/>
@@ -1724,16 +1724,16 @@
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>Informatievoorziening</v>
+        <v>Sociaal Domein</v>
       </c>
       <c r="B58" t="str">
-        <v>Proces</v>
+        <v>Mens</v>
       </c>
       <c r="C58" t="str">
-        <v>roadmap-transparantie</v>
+        <v>capaciteit-kennis</v>
       </c>
       <c r="D58" t="str">
-        <v>De productroadmap is transparant, realistisch en sluit aan bij NDS-prioriteiten en gemeentelijke behoeften</v>
+        <v>De personele capaciteit (aantal en kennisniveau) is op orde om producten te ondersteunen en door te ontwikkelen en heeft een meerjaars forecast</v>
       </c>
       <c r="E58" t="str">
         <v/>
@@ -1747,19 +1747,19 @@
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>Informatievoorziening</v>
+        <v>Sociaal Domein</v>
       </c>
       <c r="B59" t="str">
-        <v>Proces</v>
+        <v>Mens</v>
       </c>
       <c r="C59" t="str">
-        <v>burgers-ondernemers-centraal</v>
+        <v>digitaal-vakmanschap</v>
       </c>
       <c r="D59" t="str">
-        <v>De producten stellen gemeenten in staat burgers en ondernemers als één overheid te bedienen met geïntegreerde digitale dienstverlening</v>
+        <v>PinkRoccade investeert aantoonbaar in kennisontwikkeling (nieuwe technologieën, AI, Common Ground) en ondersteunt gemeenten hierbij</v>
       </c>
       <c r="E59" t="str">
-        <v>Burgers en ondernemers centraal</v>
+        <v>Digitaal vakmanschap</v>
       </c>
       <c r="F59" t="str">
         <v/>
@@ -1770,16 +1770,16 @@
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>Informatievoorziening</v>
+        <v>Sociaal Domein</v>
       </c>
       <c r="B60" t="str">
-        <v>Proces</v>
+        <v>Mens</v>
       </c>
       <c r="C60" t="str">
-        <v>prijsbeleid</v>
+        <v>klantbetrokkenheid</v>
       </c>
       <c r="D60" t="str">
-        <v>Prijsbeleid (inclusief offertes) is uitlegbaar en marktconform en hanteert een voorspelbaar proces</v>
+        <v>Gebruikers worden structureel betrokken bij doorontwikkeling (co-creatie, klankbordgroepen, roadmap-invloed) en de betrokkenheid wordt op kwaliteit en kwantiteit periodiek geëvalueerd</v>
       </c>
       <c r="E60" t="str">
         <v/>
@@ -1793,30 +1793,605 @@
     </row>
     <row r="61">
       <c r="A61" t="str">
+        <v>Sociaal Domein</v>
+      </c>
+      <c r="B61" t="str">
+        <v>Mens</v>
+      </c>
+      <c r="C61" t="str">
+        <v>opleiding-continuiteit</v>
+      </c>
+      <c r="D61" t="str">
+        <v>Training, documentatie en support zijn op orde; kennisborging is geborgd en niet afhankelijk van individuen</v>
+      </c>
+      <c r="E61" t="str">
+        <v/>
+      </c>
+      <c r="F61" t="str">
+        <v/>
+      </c>
+      <c r="G61" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="str">
+        <v>Sociaal Domein</v>
+      </c>
+      <c r="B62" t="str">
+        <v>Proces</v>
+      </c>
+      <c r="C62" t="str">
+        <v>dienstverlening-nps</v>
+      </c>
+      <c r="D62" t="str">
+        <v>De dienstverlening is uniform tussen businessunits; NPS en klanttevredenheid worden structureel gemeten en vertaald naar verbeteracties en gepubliceerd</v>
+      </c>
+      <c r="E62" t="str">
+        <v/>
+      </c>
+      <c r="F62" t="str">
+        <v/>
+      </c>
+      <c r="G62" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="str">
+        <v>Sociaal Domein</v>
+      </c>
+      <c r="B63" t="str">
+        <v>Proces</v>
+      </c>
+      <c r="C63" t="str">
+        <v>release-incident</v>
+      </c>
+      <c r="D63" t="str">
+        <v>Releases zijn voorspelbaar en goed gecommuniceerd; incidenten worden snel en transparant conform SLA afgehandeld</v>
+      </c>
+      <c r="E63" t="str">
+        <v/>
+      </c>
+      <c r="F63" t="str">
+        <v/>
+      </c>
+      <c r="G63" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="str">
+        <v>Sociaal Domein</v>
+      </c>
+      <c r="B64" t="str">
+        <v>Proces</v>
+      </c>
+      <c r="C64" t="str">
+        <v>roadmap-transparantie</v>
+      </c>
+      <c r="D64" t="str">
+        <v>De productroadmap is transparant, realistisch en sluit aan bij NDS-prioriteiten en gemeentelijke behoeften</v>
+      </c>
+      <c r="E64" t="str">
+        <v/>
+      </c>
+      <c r="F64" t="str">
+        <v/>
+      </c>
+      <c r="G64" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="str">
+        <v>Sociaal Domein</v>
+      </c>
+      <c r="B65" t="str">
+        <v>Proces</v>
+      </c>
+      <c r="C65" t="str">
+        <v>burgers-ondernemers-centraal</v>
+      </c>
+      <c r="D65" t="str">
+        <v>De producten stellen gemeenten in staat burgers en ondernemers als één overheid te bedienen met geïntegreerde digitale dienstverlening</v>
+      </c>
+      <c r="E65" t="str">
+        <v>Burgers en ondernemers centraal</v>
+      </c>
+      <c r="F65" t="str">
+        <v/>
+      </c>
+      <c r="G65" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="str">
+        <v>Sociaal Domein</v>
+      </c>
+      <c r="B66" t="str">
+        <v>Proces</v>
+      </c>
+      <c r="C66" t="str">
+        <v>prijsbeleid</v>
+      </c>
+      <c r="D66" t="str">
+        <v>Prijsbeleid (inclusief offertes) is uitlegbaar en marktconform en hanteert een voorspelbaar proces</v>
+      </c>
+      <c r="E66" t="str">
+        <v/>
+      </c>
+      <c r="F66" t="str">
+        <v/>
+      </c>
+      <c r="G66" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="str">
+        <v>Sociaal Domein</v>
+      </c>
+      <c r="B67" t="str">
+        <v>Proces</v>
+      </c>
+      <c r="C67" t="str">
+        <v>lifecyclemanagement</v>
+      </c>
+      <c r="D67" t="str">
+        <v>Lifecyclemanagement volgt de afspraken van de uitvloeiingsregeling</v>
+      </c>
+      <c r="E67" t="str">
+        <v/>
+      </c>
+      <c r="F67" t="str">
+        <v/>
+      </c>
+      <c r="G67" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="str">
+        <v>Sociaal Domein</v>
+      </c>
+      <c r="B68" t="str">
+        <v>Proces</v>
+      </c>
+      <c r="C68" t="str">
+        <v>partner-productontwikkeling</v>
+      </c>
+      <c r="D68" t="str">
+        <v>PinkRoccade is een partner van betekenis: de productontwikkeling sluit voldoende aan bij de wensen en eisen die vanuit de markt (gemeenten) worden gesteld</v>
+      </c>
+      <c r="E68" t="str">
+        <v/>
+      </c>
+      <c r="F68" t="str">
+        <v/>
+      </c>
+      <c r="G68" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="str">
+        <v>Sociaal Domein</v>
+      </c>
+      <c r="B69" t="str">
+        <v>Proces</v>
+      </c>
+      <c r="C69" t="str">
+        <v>partner-dienstverlening</v>
+      </c>
+      <c r="D69" t="str">
+        <v>PinkRoccade is een partner van betekenis: de dienstverlening sluit voldoende aan bij de wensen en eisen die vanuit de markt (gemeenten) worden gesteld</v>
+      </c>
+      <c r="E69" t="str">
+        <v/>
+      </c>
+      <c r="F69" t="str">
+        <v/>
+      </c>
+      <c r="G69" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="str">
         <v>Informatievoorziening</v>
       </c>
-      <c r="B61" t="str">
-        <v>Proces</v>
-      </c>
-      <c r="C61" t="str">
+      <c r="B70" t="str">
+        <v/>
+      </c>
+      <c r="C70" t="str">
+        <v/>
+      </c>
+      <c r="D70" t="str">
+        <v/>
+      </c>
+      <c r="E70" t="str">
+        <v/>
+      </c>
+      <c r="F70" t="str">
+        <v/>
+      </c>
+      <c r="G70" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="str">
+        <v>Informatievoorziening</v>
+      </c>
+      <c r="B71" t="str">
+        <v>Techniek</v>
+      </c>
+      <c r="C71" t="str">
+        <v>common-ground-standaarden</v>
+      </c>
+      <c r="D71" t="str">
+        <v>De producten voldoen aan Common Ground-principes en open standaarden (API-first, ZGW-API's, iConnect, scheiding data/logica)</v>
+      </c>
+      <c r="E71" t="str">
+        <v>Open</v>
+      </c>
+      <c r="F71" t="str">
+        <v/>
+      </c>
+      <c r="G71" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="str">
+        <v>Informatievoorziening</v>
+      </c>
+      <c r="B72" t="str">
+        <v>Techniek</v>
+      </c>
+      <c r="C72" t="str">
+        <v>cloud-data</v>
+      </c>
+      <c r="D72" t="str">
+        <v>De producten zijn volwaardige SaaS-oplossingen met datagedreven werken: data via API's beschikbaar voor analyse en veilig deelbaar over overheidslagen</v>
+      </c>
+      <c r="E72" t="str">
+        <v>Cloud</v>
+      </c>
+      <c r="F72" t="str">
+        <v/>
+      </c>
+      <c r="G72" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="str">
+        <v>Informatievoorziening</v>
+      </c>
+      <c r="B73" t="str">
+        <v>Techniek</v>
+      </c>
+      <c r="C73" t="str">
+        <v>ai-integratie</v>
+      </c>
+      <c r="D73" t="str">
+        <v>AI is concreet en bruikbaar onderdeel van de productportfolio (werkende functionaliteit, niet alleen visie) en hierover zijn risicoanalyses uitgevoerd en een AI-act assessment van beschikbaar</v>
+      </c>
+      <c r="E73" t="str">
+        <v>AI</v>
+      </c>
+      <c r="F73" t="str">
+        <v/>
+      </c>
+      <c r="G73" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="str">
+        <v>Informatievoorziening</v>
+      </c>
+      <c r="B74" t="str">
+        <v>Techniek</v>
+      </c>
+      <c r="C74" t="str">
+        <v>digitale-weerbaarheid</v>
+      </c>
+      <c r="D74" t="str">
+        <v>De producten voldoen aan actuele security-eisen (BIO, NIS2, pentesting) en verminderen leveranciersafhankelijkheid</v>
+      </c>
+      <c r="E74" t="str">
+        <v>Digitale weerbaarheid en autonomie</v>
+      </c>
+      <c r="F74" t="str">
+        <v/>
+      </c>
+      <c r="G74" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="str">
+        <v>Informatievoorziening</v>
+      </c>
+      <c r="B75" t="str">
+        <v>Mens</v>
+      </c>
+      <c r="C75" t="str">
+        <v>capaciteit-kennis</v>
+      </c>
+      <c r="D75" t="str">
+        <v>De personele capaciteit (aantal en kennisniveau) is op orde om producten te ondersteunen en door te ontwikkelen en heeft een meerjaars forecast</v>
+      </c>
+      <c r="E75" t="str">
+        <v/>
+      </c>
+      <c r="F75" t="str">
+        <v/>
+      </c>
+      <c r="G75" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="str">
+        <v>Informatievoorziening</v>
+      </c>
+      <c r="B76" t="str">
+        <v>Mens</v>
+      </c>
+      <c r="C76" t="str">
+        <v>digitaal-vakmanschap</v>
+      </c>
+      <c r="D76" t="str">
+        <v>PinkRoccade investeert aantoonbaar in kennisontwikkeling (nieuwe technologieën, AI, Common Ground) en ondersteunt gemeenten hierbij</v>
+      </c>
+      <c r="E76" t="str">
+        <v>Digitaal vakmanschap</v>
+      </c>
+      <c r="F76" t="str">
+        <v/>
+      </c>
+      <c r="G76" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="str">
+        <v>Informatievoorziening</v>
+      </c>
+      <c r="B77" t="str">
+        <v>Mens</v>
+      </c>
+      <c r="C77" t="str">
+        <v>klantbetrokkenheid</v>
+      </c>
+      <c r="D77" t="str">
+        <v>Gebruikers worden structureel betrokken bij doorontwikkeling (co-creatie, klankbordgroepen, roadmap-invloed) en de betrokkenheid wordt op kwaliteit en kwantiteit periodiek geëvalueerd</v>
+      </c>
+      <c r="E77" t="str">
+        <v/>
+      </c>
+      <c r="F77" t="str">
+        <v/>
+      </c>
+      <c r="G77" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="str">
+        <v>Informatievoorziening</v>
+      </c>
+      <c r="B78" t="str">
+        <v>Mens</v>
+      </c>
+      <c r="C78" t="str">
+        <v>opleiding-continuiteit</v>
+      </c>
+      <c r="D78" t="str">
+        <v>Training, documentatie en support zijn op orde; kennisborging is geborgd en niet afhankelijk van individuen</v>
+      </c>
+      <c r="E78" t="str">
+        <v/>
+      </c>
+      <c r="F78" t="str">
+        <v/>
+      </c>
+      <c r="G78" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="str">
+        <v>Informatievoorziening</v>
+      </c>
+      <c r="B79" t="str">
+        <v>Proces</v>
+      </c>
+      <c r="C79" t="str">
+        <v>dienstverlening-nps</v>
+      </c>
+      <c r="D79" t="str">
+        <v>De dienstverlening is uniform tussen businessunits; NPS en klanttevredenheid worden structureel gemeten en vertaald naar verbeteracties en gepubliceerd</v>
+      </c>
+      <c r="E79" t="str">
+        <v/>
+      </c>
+      <c r="F79" t="str">
+        <v/>
+      </c>
+      <c r="G79" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="str">
+        <v>Informatievoorziening</v>
+      </c>
+      <c r="B80" t="str">
+        <v>Proces</v>
+      </c>
+      <c r="C80" t="str">
+        <v>release-incident</v>
+      </c>
+      <c r="D80" t="str">
+        <v>Releases zijn voorspelbaar en goed gecommuniceerd; incidenten worden snel en transparant conform SLA afgehandeld</v>
+      </c>
+      <c r="E80" t="str">
+        <v/>
+      </c>
+      <c r="F80" t="str">
+        <v/>
+      </c>
+      <c r="G80" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="str">
+        <v>Informatievoorziening</v>
+      </c>
+      <c r="B81" t="str">
+        <v>Proces</v>
+      </c>
+      <c r="C81" t="str">
+        <v>roadmap-transparantie</v>
+      </c>
+      <c r="D81" t="str">
+        <v>De productroadmap is transparant, realistisch en sluit aan bij NDS-prioriteiten en gemeentelijke behoeften</v>
+      </c>
+      <c r="E81" t="str">
+        <v/>
+      </c>
+      <c r="F81" t="str">
+        <v/>
+      </c>
+      <c r="G81" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="str">
+        <v>Informatievoorziening</v>
+      </c>
+      <c r="B82" t="str">
+        <v>Proces</v>
+      </c>
+      <c r="C82" t="str">
+        <v>burgers-ondernemers-centraal</v>
+      </c>
+      <c r="D82" t="str">
+        <v>De producten stellen gemeenten in staat burgers en ondernemers als één overheid te bedienen met geïntegreerde digitale dienstverlening</v>
+      </c>
+      <c r="E82" t="str">
+        <v>Burgers en ondernemers centraal</v>
+      </c>
+      <c r="F82" t="str">
+        <v/>
+      </c>
+      <c r="G82" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="str">
+        <v>Informatievoorziening</v>
+      </c>
+      <c r="B83" t="str">
+        <v>Proces</v>
+      </c>
+      <c r="C83" t="str">
+        <v>prijsbeleid</v>
+      </c>
+      <c r="D83" t="str">
+        <v>Prijsbeleid (inclusief offertes) is uitlegbaar en marktconform en hanteert een voorspelbaar proces</v>
+      </c>
+      <c r="E83" t="str">
+        <v/>
+      </c>
+      <c r="F83" t="str">
+        <v/>
+      </c>
+      <c r="G83" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="str">
+        <v>Informatievoorziening</v>
+      </c>
+      <c r="B84" t="str">
+        <v>Proces</v>
+      </c>
+      <c r="C84" t="str">
         <v>lifecyclemanagement</v>
       </c>
-      <c r="D61" t="str">
+      <c r="D84" t="str">
         <v>Lifecyclemanagement volgt de afspraken van de uitvloeiingsregeling</v>
       </c>
-      <c r="E61" t="str">
-        <v/>
-      </c>
-      <c r="F61" t="str">
-        <v/>
-      </c>
-      <c r="G61" t="str">
+      <c r="E84" t="str">
+        <v/>
+      </c>
+      <c r="F84" t="str">
+        <v/>
+      </c>
+      <c r="G84" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="str">
+        <v>Informatievoorziening</v>
+      </c>
+      <c r="B85" t="str">
+        <v>Proces</v>
+      </c>
+      <c r="C85" t="str">
+        <v>partner-productontwikkeling</v>
+      </c>
+      <c r="D85" t="str">
+        <v>PinkRoccade is een partner van betekenis: de productontwikkeling sluit voldoende aan bij de wensen en eisen die vanuit de markt (gemeenten) worden gesteld</v>
+      </c>
+      <c r="E85" t="str">
+        <v/>
+      </c>
+      <c r="F85" t="str">
+        <v/>
+      </c>
+      <c r="G85" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="str">
+        <v>Informatievoorziening</v>
+      </c>
+      <c r="B86" t="str">
+        <v>Proces</v>
+      </c>
+      <c r="C86" t="str">
+        <v>partner-dienstverlening</v>
+      </c>
+      <c r="D86" t="str">
+        <v>PinkRoccade is een partner van betekenis: de dienstverlening sluit voldoende aan bij de wensen en eisen die vanuit de markt (gemeenten) worden gesteld</v>
+      </c>
+      <c r="E86" t="str">
+        <v/>
+      </c>
+      <c r="F86" t="str">
+        <v/>
+      </c>
+      <c r="G86" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G61"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G86"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1846,10 +2421,10 @@
         <v>1</v>
       </c>
       <c r="B2" t="str">
-        <v>Afwezig</v>
+        <v>Initial</v>
       </c>
       <c r="C2" t="str">
-        <v>Er is niets van zichtbaar</v>
+        <v>Ad-hoc, geen gestructureerde aanpak</v>
       </c>
     </row>
     <row r="3">
@@ -1857,10 +2432,10 @@
         <v>2</v>
       </c>
       <c r="B3" t="str">
-        <v>Initieel</v>
+        <v>Managed</v>
       </c>
       <c r="C3" t="str">
-        <v>Ad hoc, niet structureel</v>
+        <v>Herhaalbaar op projectniveau, nog niet organisatiebreed geborgd</v>
       </c>
     </row>
     <row r="4">
@@ -1868,10 +2443,10 @@
         <v>3</v>
       </c>
       <c r="B4" t="str">
-        <v>Herhaalbaar</v>
+        <v>Defined</v>
       </c>
       <c r="C4" t="str">
-        <v>Er is een aanpak maar niet consistent</v>
+        <v>Gestandaardiseerd en organisatiebreed vastgelegd</v>
       </c>
     </row>
     <row r="5">
@@ -1879,10 +2454,10 @@
         <v>4</v>
       </c>
       <c r="B5" t="str">
-        <v>Gedefinieerd</v>
+        <v>Quantitatively Managed</v>
       </c>
       <c r="C5" t="str">
-        <v>Structureel ingericht en meetbaar</v>
+        <v>Gemeten en gestuurd op basis van data</v>
       </c>
     </row>
     <row r="6">
@@ -1890,10 +2465,10 @@
         <v>5</v>
       </c>
       <c r="B6" t="str">
-        <v>Best practice</v>
+        <v>Optimizing</v>
       </c>
       <c r="C6" t="str">
-        <v>Voorbeeldstellend, continu verbeterend</v>
+        <v>Continue verbetering ingebed in de organisatie</v>
       </c>
     </row>
   </sheetData>
@@ -1976,7 +2551,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:B6"/>
   <cols>
     <col min="1" max="1" width="25.83203125" customWidth="1"/>
     <col min="2" max="2" width="25.83203125" customWidth="1"/>
@@ -2000,31 +2575,39 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>burgerzaken</v>
+        <v>ro</v>
       </c>
       <c r="B3" t="str">
-        <v>Burgerzaken</v>
+        <v>R&amp;O</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>sociaal-domein</v>
+        <v>burgerzaken</v>
       </c>
       <c r="B4" t="str">
-        <v>Sociaal Domein</v>
+        <v>Burgerzaken</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
+        <v>sociaal-domein</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Sociaal Domein</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
         <v>informatievoorziening</v>
       </c>
-      <c r="B5" t="str">
+      <c r="B6" t="str">
         <v>Informatievoorziening</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B6"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>